<commit_message>
Thu 23 Apr 2026 16:42:21 EDT
</commit_message>
<xml_diff>
--- a/machine_learning/injection/DDLUCJ-experiment-pipeline/repostprocess.xlsx
+++ b/machine_learning/injection/DDLUCJ-experiment-pipeline/repostprocess.xlsx
@@ -1173,13 +1173,13 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>-213.1797011444954</v>
+        <v>-212.5076523839172</v>
       </c>
       <c r="H17" t="n">
         <v>9</v>
       </c>
       <c r="I17" t="n">
-        <v>163.9126653559515</v>
+        <v>835.9614259341015</v>
       </c>
       <c r="J17" t="n">
         <v>-213.3436138098513</v>
@@ -1569,13 +1569,13 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>-213.2010260388874</v>
+        <v>-213.1913236081741</v>
       </c>
       <c r="H26" t="n">
         <v>9</v>
       </c>
       <c r="I26" t="n">
-        <v>142.5877709638712</v>
+        <v>152.2902016772605</v>
       </c>
       <c r="J26" t="n">
         <v>-213.3436138098513</v>
@@ -1613,13 +1613,13 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>-213.1576975976407</v>
+        <v>-213.1453605980934</v>
       </c>
       <c r="H27" t="n">
         <v>9</v>
       </c>
       <c r="I27" t="n">
-        <v>185.9162122106</v>
+        <v>198.2532117579581</v>
       </c>
       <c r="J27" t="n">
         <v>-213.3436138098513</v>
@@ -1657,13 +1657,13 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>-213.1494842471058</v>
+        <v>-213.1421481222368</v>
       </c>
       <c r="H28" t="n">
         <v>9</v>
       </c>
       <c r="I28" t="n">
-        <v>194.1295627455588</v>
+        <v>201.4656876145295</v>
       </c>
       <c r="J28" t="n">
         <v>-213.3436138098513</v>
@@ -1701,13 +1701,13 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>-213.1768401791302</v>
+        <v>-213.1504876770753</v>
       </c>
       <c r="H29" t="n">
         <v>9</v>
       </c>
       <c r="I29" t="n">
-        <v>166.7736307211385</v>
+        <v>193.1261327760581</v>
       </c>
       <c r="J29" t="n">
         <v>-213.3436138098513</v>
@@ -1745,13 +1745,13 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>-213.2021082851193</v>
+        <v>-213.2021082851187</v>
       </c>
       <c r="H30" t="n">
         <v>9</v>
       </c>
       <c r="I30" t="n">
-        <v>141.5055247320538</v>
+        <v>141.5055247326222</v>
       </c>
       <c r="J30" t="n">
         <v>-213.3436138098513</v>
@@ -1789,13 +1789,13 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>-213.3262251973137</v>
+        <v>-213.3245633351582</v>
       </c>
       <c r="H31" t="n">
         <v>9</v>
       </c>
       <c r="I31" t="n">
-        <v>17.3886125376157</v>
+        <v>19.05047469307419</v>
       </c>
       <c r="J31" t="n">
         <v>-213.3436138098513</v>
@@ -1833,13 +1833,13 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>-215.968055814278</v>
+        <v>-214.7028624898805</v>
       </c>
       <c r="H32" t="n">
         <v>9</v>
       </c>
       <c r="I32" t="n">
-        <v>-17.64427274508762</v>
+        <v>1247.549051652413</v>
       </c>
       <c r="J32" t="n">
         <v>-215.950411541533</v>
@@ -2933,13 +2933,13 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>-215.9581723862323</v>
+        <v>-215.9561682360744</v>
       </c>
       <c r="H57" t="n">
         <v>9</v>
       </c>
       <c r="I57" t="n">
-        <v>39.84627146732578</v>
+        <v>41.85042162518471</v>
       </c>
       <c r="J57" t="n">
         <v>-215.9980186576996</v>
@@ -3021,13 +3021,13 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>-215.9644015486025</v>
+        <v>-215.9589175726923</v>
       </c>
       <c r="H59" t="n">
         <v>9</v>
       </c>
       <c r="I59" t="n">
-        <v>33.61710909709359</v>
+        <v>39.10108500727461</v>
       </c>
       <c r="J59" t="n">
         <v>-215.9980186576996</v>
@@ -3109,13 +3109,13 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>-215.9650296003272</v>
+        <v>-215.9462074712169</v>
       </c>
       <c r="H61" t="n">
         <v>9</v>
       </c>
       <c r="I61" t="n">
-        <v>32.98905737241853</v>
+        <v>51.81118648269489</v>
       </c>
       <c r="J61" t="n">
         <v>-215.9980186576996</v>
@@ -3153,13 +3153,13 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>-215.9927398868854</v>
+        <v>-215.9924367471406</v>
       </c>
       <c r="H62" t="n">
         <v>9</v>
       </c>
       <c r="I62" t="n">
-        <v>5.278770814214795</v>
+        <v>5.58191055895918</v>
       </c>
       <c r="J62" t="n">
         <v>-215.9980186576996</v>
@@ -4825,13 +4825,13 @@
         </is>
       </c>
       <c r="G100" t="n">
-        <v>-154.0374616701789</v>
+        <v>-152.5516160270816</v>
       </c>
       <c r="H100" t="n">
         <v>10</v>
       </c>
       <c r="I100" t="n">
-        <v>880.4808055724038</v>
+        <v>2366.326448669724</v>
       </c>
       <c r="J100" t="n">
         <v>-154.9179424757513</v>
@@ -6805,13 +6805,13 @@
         </is>
       </c>
       <c r="G145" t="n">
-        <v>-152.4172048110165</v>
+        <v>-150.9927345104938</v>
       </c>
       <c r="H145" t="n">
         <v>10</v>
       </c>
       <c r="I145" t="n">
-        <v>888.2046307869587</v>
+        <v>2312.67493130963</v>
       </c>
       <c r="J145" t="n">
         <v>-153.3054094418034</v>
@@ -7685,13 +7685,13 @@
         </is>
       </c>
       <c r="G165" t="n">
-        <v>-154.9418518681631</v>
+        <v>-153.2907289076241</v>
       </c>
       <c r="H165" t="n">
         <v>10</v>
       </c>
       <c r="I165" t="n">
-        <v>8.77657079678329</v>
+        <v>1659.899531335782</v>
       </c>
       <c r="J165" t="n">
         <v>-154.9506284389599</v>
@@ -8169,13 +8169,13 @@
         </is>
       </c>
       <c r="G176" t="n">
-        <v>-154.9428967494533</v>
+        <v>-153.6477628265835</v>
       </c>
       <c r="H176" t="n">
         <v>10</v>
       </c>
       <c r="I176" t="n">
-        <v>7.731689506613293</v>
+        <v>1302.865612376422</v>
       </c>
       <c r="J176" t="n">
         <v>-154.9506284389599</v>
@@ -9093,13 +9093,13 @@
         </is>
       </c>
       <c r="G197" t="n">
-        <v>-154.9357737754797</v>
+        <v>-153.8618972276274</v>
       </c>
       <c r="H197" t="n">
         <v>10</v>
       </c>
       <c r="I197" t="n">
-        <v>79.67717566805277</v>
+        <v>1153.553723520361</v>
       </c>
       <c r="J197" t="n">
         <v>-155.0154509511478</v>
@@ -9753,13 +9753,13 @@
         </is>
       </c>
       <c r="G212" t="n">
-        <v>-154.1883851378736</v>
+        <v>-153.7263205808158</v>
       </c>
       <c r="H212" t="n">
         <v>10</v>
       </c>
       <c r="I212" t="n">
-        <v>827.065813274146</v>
+        <v>1289.130370331975</v>
       </c>
       <c r="J212" t="n">
         <v>-155.0154509511478</v>
@@ -15175,13 +15175,13 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>-191.9517670449475</v>
+        <v>-190.9183003641962</v>
       </c>
       <c r="H333" t="n">
         <v>10</v>
       </c>
       <c r="I333" t="n">
-        <v>2.004920530794152</v>
+        <v>1035.471601282154</v>
       </c>
       <c r="J333" t="n">
         <v>-191.9537719654783</v>

</xml_diff>

<commit_message>
Thu  7 May 2026 17:11:51 EDT figures
</commit_message>
<xml_diff>
--- a/machine_learning/injection/DDLUCJ-experiment-pipeline/repostprocess.xlsx
+++ b/machine_learning/injection/DDLUCJ-experiment-pipeline/repostprocess.xlsx
@@ -519,13 +519,13 @@
         <v>9</v>
       </c>
       <c r="I2" t="n">
-        <v>174.6675498512786</v>
+        <v>174.6675498513071</v>
       </c>
       <c r="J2" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K2" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L2" t="inlineStr"/>
     </row>
@@ -563,13 +563,13 @@
         <v>9</v>
       </c>
       <c r="I3" t="n">
-        <v>161.9892498513025</v>
+        <v>161.9892498513309</v>
       </c>
       <c r="J3" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K3" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
@@ -607,13 +607,13 @@
         <v>9</v>
       </c>
       <c r="I4" t="n">
-        <v>148.4081798512875</v>
+        <v>148.4081798513159</v>
       </c>
       <c r="J4" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K4" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
@@ -651,13 +651,13 @@
         <v>9</v>
       </c>
       <c r="I5" t="n">
-        <v>87.87446985130032</v>
+        <v>87.87446985132874</v>
       </c>
       <c r="J5" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K5" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L5" t="inlineStr"/>
     </row>
@@ -695,13 +695,13 @@
         <v>9</v>
       </c>
       <c r="I6" t="n">
-        <v>183.2405498512912</v>
+        <v>183.2405498513197</v>
       </c>
       <c r="J6" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K6" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L6" t="inlineStr"/>
     </row>
@@ -739,13 +739,13 @@
         <v>9</v>
       </c>
       <c r="I7" t="n">
-        <v>78.88592985128184</v>
+        <v>78.88592985131027</v>
       </c>
       <c r="J7" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K7" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
@@ -783,13 +783,13 @@
         <v>9</v>
       </c>
       <c r="I8" t="n">
-        <v>208.2775198512934</v>
+        <v>208.2775198513218</v>
       </c>
       <c r="J8" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K8" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
@@ -827,13 +827,13 @@
         <v>9</v>
       </c>
       <c r="I9" t="n">
-        <v>203.7836098512855</v>
+        <v>203.7836098513139</v>
       </c>
       <c r="J9" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K9" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
@@ -871,13 +871,13 @@
         <v>9</v>
       </c>
       <c r="I10" t="n">
-        <v>205.4438198512969</v>
+        <v>205.4438198513253</v>
       </c>
       <c r="J10" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K10" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L10" t="inlineStr"/>
     </row>
@@ -915,13 +915,13 @@
         <v>9</v>
       </c>
       <c r="I11" t="n">
-        <v>196.59118985129</v>
+        <v>196.5911898513184</v>
       </c>
       <c r="J11" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K11" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
@@ -959,13 +959,13 @@
         <v>9</v>
       </c>
       <c r="I12" t="n">
-        <v>179.3521498512973</v>
+        <v>179.3521498513257</v>
       </c>
       <c r="J12" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K12" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
@@ -1003,13 +1003,13 @@
         <v>9</v>
       </c>
       <c r="I13" t="n">
-        <v>47.68020985127919</v>
+        <v>47.68020985130761</v>
       </c>
       <c r="J13" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K13" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
@@ -1047,13 +1047,13 @@
         <v>9</v>
       </c>
       <c r="I14" t="n">
-        <v>212.9298998513036</v>
+        <v>212.929899851332</v>
       </c>
       <c r="J14" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K14" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
@@ -1091,13 +1091,13 @@
         <v>9</v>
       </c>
       <c r="I15" t="n">
-        <v>212.0808798512996</v>
+        <v>212.0808798513281</v>
       </c>
       <c r="J15" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K15" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
@@ -1135,13 +1135,13 @@
         <v>9</v>
       </c>
       <c r="I16" t="n">
-        <v>201.4672698512925</v>
+        <v>201.4672698513209</v>
       </c>
       <c r="J16" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K16" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
@@ -1179,13 +1179,13 @@
         <v>9</v>
       </c>
       <c r="I17" t="n">
-        <v>202.7135898512995</v>
+        <v>202.7135898513279</v>
       </c>
       <c r="J17" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K17" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
@@ -1223,13 +1223,13 @@
         <v>9</v>
       </c>
       <c r="I18" t="n">
-        <v>206.2314398512797</v>
+        <v>206.2314398513081</v>
       </c>
       <c r="J18" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K18" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
@@ -1267,13 +1267,13 @@
         <v>9</v>
       </c>
       <c r="I19" t="n">
-        <v>40.96755985128198</v>
+        <v>40.9675598513104</v>
       </c>
       <c r="J19" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K19" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
@@ -1311,13 +1311,13 @@
         <v>9</v>
       </c>
       <c r="I20" t="n">
-        <v>213.8370098512894</v>
+        <v>213.8370098513178</v>
       </c>
       <c r="J20" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K20" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
@@ -1355,13 +1355,13 @@
         <v>9</v>
       </c>
       <c r="I21" t="n">
-        <v>203.2361698512943</v>
+        <v>203.2361698513228</v>
       </c>
       <c r="J21" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K21" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
@@ -1399,13 +1399,13 @@
         <v>9</v>
       </c>
       <c r="I22" t="n">
-        <v>217.948019851292</v>
+        <v>217.9480198513204</v>
       </c>
       <c r="J22" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K22" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
@@ -1443,13 +1443,13 @@
         <v>9</v>
       </c>
       <c r="I23" t="n">
-        <v>216.5417398512943</v>
+        <v>216.5417398513227</v>
       </c>
       <c r="J23" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K23" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
@@ -1487,13 +1487,13 @@
         <v>9</v>
       </c>
       <c r="I24" t="n">
-        <v>207.1036798512864</v>
+        <v>207.1036798513148</v>
       </c>
       <c r="J24" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K24" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
@@ -1531,13 +1531,13 @@
         <v>9</v>
       </c>
       <c r="I25" t="n">
-        <v>43.38156985127739</v>
+        <v>43.38156985130581</v>
       </c>
       <c r="J25" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K25" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
@@ -1575,13 +1575,13 @@
         <v>9</v>
       </c>
       <c r="I26" t="n">
-        <v>209.8763998512823</v>
+        <v>209.8763998513107</v>
       </c>
       <c r="J26" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K26" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
@@ -1619,13 +1619,13 @@
         <v>9</v>
       </c>
       <c r="I27" t="n">
-        <v>173.5600798512849</v>
+        <v>173.5600798513133</v>
       </c>
       <c r="J27" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K27" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
@@ -1663,13 +1663,13 @@
         <v>9</v>
       </c>
       <c r="I28" t="n">
-        <v>215.7015198512795</v>
+        <v>215.7015198513079</v>
       </c>
       <c r="J28" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K28" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
@@ -1707,13 +1707,13 @@
         <v>9</v>
       </c>
       <c r="I29" t="n">
-        <v>186.4891198513021</v>
+        <v>186.4891198513305</v>
       </c>
       <c r="J29" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K29" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
@@ -1751,13 +1751,13 @@
         <v>9</v>
       </c>
       <c r="I30" t="n">
-        <v>209.6131698512806</v>
+        <v>209.6131698513091</v>
       </c>
       <c r="J30" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K30" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
@@ -1795,13 +1795,13 @@
         <v>9</v>
       </c>
       <c r="I31" t="n">
-        <v>71.63411985129642</v>
+        <v>71.63411985132484</v>
       </c>
       <c r="J31" t="n">
         <v>-213.3436138098513</v>
       </c>
       <c r="K31" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
@@ -5859,10 +5859,10 @@
         <v>4</v>
       </c>
       <c r="I122" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J122" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K122" t="n">
         <v>-56.20522331321214</v>
@@ -5905,10 +5905,10 @@
         <v>4</v>
       </c>
       <c r="I123" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J123" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K123" t="n">
         <v>-56.20522331321214</v>
@@ -5951,10 +5951,10 @@
         <v>4</v>
       </c>
       <c r="I124" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J124" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K124" t="n">
         <v>-56.20522331321214</v>
@@ -5997,10 +5997,10 @@
         <v>4</v>
       </c>
       <c r="I125" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J125" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K125" t="n">
         <v>-56.20522331321214</v>
@@ -6043,10 +6043,10 @@
         <v>4</v>
       </c>
       <c r="I126" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J126" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K126" t="n">
         <v>-56.20522331321214</v>
@@ -6089,10 +6089,10 @@
         <v>4</v>
       </c>
       <c r="I127" t="n">
-        <v>-0.002214823119572884</v>
+        <v>-0.002214823126678311</v>
       </c>
       <c r="J127" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K127" t="n">
         <v>-56.20522331321214</v>
@@ -6135,10 +6135,10 @@
         <v>4</v>
       </c>
       <c r="I128" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J128" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K128" t="n">
         <v>-56.20522331321214</v>
@@ -6181,10 +6181,10 @@
         <v>4</v>
       </c>
       <c r="I129" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J129" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K129" t="n">
         <v>-56.20522331321214</v>
@@ -6227,10 +6227,10 @@
         <v>4</v>
       </c>
       <c r="I130" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J130" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K130" t="n">
         <v>-56.20522331321214</v>
@@ -6273,10 +6273,10 @@
         <v>4</v>
       </c>
       <c r="I131" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J131" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K131" t="n">
         <v>-56.20522331321214</v>
@@ -6319,10 +6319,10 @@
         <v>4</v>
       </c>
       <c r="I132" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J132" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K132" t="n">
         <v>-56.20522331321214</v>
@@ -6365,10 +6365,10 @@
         <v>4</v>
       </c>
       <c r="I133" t="n">
-        <v>-0.002224823120400288</v>
+        <v>-0.002224823127505715</v>
       </c>
       <c r="J133" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K133" t="n">
         <v>-56.20522331321214</v>
@@ -6411,10 +6411,10 @@
         <v>4</v>
       </c>
       <c r="I134" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J134" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K134" t="n">
         <v>-56.20522331321214</v>
@@ -6457,10 +6457,10 @@
         <v>4</v>
       </c>
       <c r="I135" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J135" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K135" t="n">
         <v>-56.20522331321214</v>
@@ -6503,10 +6503,10 @@
         <v>4</v>
       </c>
       <c r="I136" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J136" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K136" t="n">
         <v>-56.20522331321214</v>
@@ -6549,10 +6549,10 @@
         <v>4</v>
       </c>
       <c r="I137" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J137" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K137" t="n">
         <v>-56.20522331321214</v>
@@ -6595,10 +6595,10 @@
         <v>4</v>
       </c>
       <c r="I138" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J138" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K138" t="n">
         <v>-56.20522331321214</v>
@@ -6641,10 +6641,10 @@
         <v>4</v>
       </c>
       <c r="I139" t="n">
-        <v>-0.002214823119572884</v>
+        <v>-0.002214823126678311</v>
       </c>
       <c r="J139" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K139" t="n">
         <v>-56.20522331321214</v>
@@ -6687,10 +6687,10 @@
         <v>4</v>
       </c>
       <c r="I140" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J140" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K140" t="n">
         <v>-56.20522331321214</v>
@@ -6733,10 +6733,10 @@
         <v>4</v>
       </c>
       <c r="I141" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J141" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K141" t="n">
         <v>-56.20522331321214</v>
@@ -6779,10 +6779,10 @@
         <v>4</v>
       </c>
       <c r="I142" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J142" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K142" t="n">
         <v>-56.20522331321214</v>
@@ -6825,10 +6825,10 @@
         <v>4</v>
       </c>
       <c r="I143" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J143" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K143" t="n">
         <v>-56.20522331321214</v>
@@ -6871,10 +6871,10 @@
         <v>4</v>
       </c>
       <c r="I144" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J144" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K144" t="n">
         <v>-56.20522331321214</v>
@@ -6917,10 +6917,10 @@
         <v>4</v>
       </c>
       <c r="I145" t="n">
-        <v>-0.002234823121227691</v>
+        <v>-0.002234823128333119</v>
       </c>
       <c r="J145" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K145" t="n">
         <v>-56.20522331321214</v>
@@ -6963,10 +6963,10 @@
         <v>4</v>
       </c>
       <c r="I146" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J146" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K146" t="n">
         <v>-56.20522331321214</v>
@@ -7009,10 +7009,10 @@
         <v>4</v>
       </c>
       <c r="I147" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J147" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K147" t="n">
         <v>-56.20522331321214</v>
@@ -7055,10 +7055,10 @@
         <v>4</v>
       </c>
       <c r="I148" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J148" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K148" t="n">
         <v>-56.20522331321214</v>
@@ -7101,10 +7101,10 @@
         <v>4</v>
       </c>
       <c r="I149" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J149" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K149" t="n">
         <v>-56.20522331321214</v>
@@ -7147,10 +7147,10 @@
         <v>4</v>
       </c>
       <c r="I150" t="n">
-        <v>-0.002244823114949668</v>
+        <v>-0.002244823122055095</v>
       </c>
       <c r="J150" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K150" t="n">
         <v>-56.20522331321214</v>
@@ -7193,10 +7193,10 @@
         <v>4</v>
       </c>
       <c r="I151" t="n">
-        <v>-0.002214823119572884</v>
+        <v>-0.002214823126678311</v>
       </c>
       <c r="J151" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="K151" t="n">
         <v>-56.20522331321214</v>
@@ -43839,10 +43839,10 @@
         <v>10</v>
       </c>
       <c r="I962" t="n">
-        <v>59.27484704275798</v>
+        <v>59.27484704270114</v>
       </c>
       <c r="J962" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K962" t="n">
         <v>-191.9364953941601</v>
@@ -43883,10 +43883,10 @@
         <v>10</v>
       </c>
       <c r="I963" t="n">
-        <v>53.05039704276737</v>
+        <v>53.05039704271053</v>
       </c>
       <c r="J963" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K963" t="n">
         <v>-191.9364953941601</v>
@@ -43927,10 +43927,10 @@
         <v>10</v>
       </c>
       <c r="I964" t="n">
-        <v>48.88530704278082</v>
+        <v>48.88530704272398</v>
       </c>
       <c r="J964" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K964" t="n">
         <v>-191.9364953941601</v>
@@ -43971,10 +43971,10 @@
         <v>10</v>
       </c>
       <c r="I965" t="n">
-        <v>35.66605704276071</v>
+        <v>35.66605704270387</v>
       </c>
       <c r="J965" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K965" t="n">
         <v>-191.9364953941601</v>
@@ -44015,10 +44015,10 @@
         <v>10</v>
       </c>
       <c r="I966" t="n">
-        <v>60.02949704276261</v>
+        <v>60.02949704270577</v>
       </c>
       <c r="J966" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K966" t="n">
         <v>-191.9364953941601</v>
@@ -44059,10 +44059,10 @@
         <v>10</v>
       </c>
       <c r="I967" t="n">
-        <v>10.13858704277482</v>
+        <v>10.13858704271797</v>
       </c>
       <c r="J967" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K967" t="n">
         <v>-191.9364953941601</v>
@@ -44103,10 +44103,10 @@
         <v>10</v>
       </c>
       <c r="I968" t="n">
-        <v>58.67554704278177</v>
+        <v>58.67554704272493</v>
       </c>
       <c r="J968" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K968" t="n">
         <v>-191.9364953941601</v>
@@ -44147,10 +44147,10 @@
         <v>10</v>
       </c>
       <c r="I969" t="n">
-        <v>59.38197704276149</v>
+        <v>59.38197704270465</v>
       </c>
       <c r="J969" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K969" t="n">
         <v>-191.9364953941601</v>
@@ -44191,10 +44191,10 @@
         <v>10</v>
       </c>
       <c r="I970" t="n">
-        <v>60.85676704276466</v>
+        <v>60.85676704270782</v>
       </c>
       <c r="J970" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K970" t="n">
         <v>-191.9364953941601</v>
@@ -44235,10 +44235,10 @@
         <v>10</v>
       </c>
       <c r="I971" t="n">
-        <v>58.72972704275981</v>
+        <v>58.72972704270296</v>
       </c>
       <c r="J971" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K971" t="n">
         <v>-191.9364953941601</v>
@@ -44279,10 +44279,10 @@
         <v>10</v>
       </c>
       <c r="I972" t="n">
-        <v>59.41868704277908</v>
+        <v>59.41868704272224</v>
       </c>
       <c r="J972" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K972" t="n">
         <v>-191.9364953941601</v>
@@ -44323,10 +44323,10 @@
         <v>10</v>
       </c>
       <c r="I973" t="n">
-        <v>28.09511704276701</v>
+        <v>28.09511704271017</v>
       </c>
       <c r="J973" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K973" t="n">
         <v>-191.9364953941601</v>
@@ -44367,10 +44367,10 @@
         <v>10</v>
       </c>
       <c r="I974" t="n">
-        <v>59.78808704276162</v>
+        <v>59.78808704270477</v>
       </c>
       <c r="J974" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K974" t="n">
         <v>-191.9364953941601</v>
@@ -44411,10 +44411,10 @@
         <v>10</v>
       </c>
       <c r="I975" t="n">
-        <v>58.48213704277327</v>
+        <v>58.48213704271643</v>
       </c>
       <c r="J975" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K975" t="n">
         <v>-191.9364953941601</v>
@@ -44455,10 +44455,10 @@
         <v>10</v>
       </c>
       <c r="I976" t="n">
-        <v>59.5360570427772</v>
+        <v>59.53605704272036</v>
       </c>
       <c r="J976" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K976" t="n">
         <v>-191.9364953941601</v>
@@ -44499,10 +44499,10 @@
         <v>10</v>
       </c>
       <c r="I977" t="n">
-        <v>58.63267704276609</v>
+        <v>58.63267704270925</v>
       </c>
       <c r="J977" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K977" t="n">
         <v>-191.9364953941601</v>
@@ -44543,10 +44543,10 @@
         <v>10</v>
       </c>
       <c r="I978" t="n">
-        <v>58.47426704278291</v>
+        <v>58.47426704272607</v>
       </c>
       <c r="J978" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K978" t="n">
         <v>-191.9364953941601</v>
@@ -44587,10 +44587,10 @@
         <v>10</v>
       </c>
       <c r="I979" t="n">
-        <v>12.0311370427828</v>
+        <v>12.03113704272596</v>
       </c>
       <c r="J979" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K979" t="n">
         <v>-191.9364953941601</v>
@@ -44631,10 +44631,10 @@
         <v>10</v>
       </c>
       <c r="I980" t="n">
-        <v>60.0741670427567</v>
+        <v>60.07416704269986</v>
       </c>
       <c r="J980" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K980" t="n">
         <v>-191.9364953941601</v>
@@ -44675,10 +44675,10 @@
         <v>10</v>
       </c>
       <c r="I981" t="n">
-        <v>58.09547704276952</v>
+        <v>58.09547704271267</v>
       </c>
       <c r="J981" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K981" t="n">
         <v>-191.9364953941601</v>
@@ -44719,10 +44719,10 @@
         <v>10</v>
       </c>
       <c r="I982" t="n">
-        <v>59.42787704276498</v>
+        <v>59.42787704270813</v>
       </c>
       <c r="J982" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K982" t="n">
         <v>-191.9364953941601</v>
@@ -44763,10 +44763,10 @@
         <v>10</v>
       </c>
       <c r="I983" t="n">
-        <v>60.19296704278077</v>
+        <v>60.19296704272392</v>
       </c>
       <c r="J983" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K983" t="n">
         <v>-191.9364953941601</v>
@@ -44807,10 +44807,10 @@
         <v>10</v>
       </c>
       <c r="I984" t="n">
-        <v>58.05750704277557</v>
+        <v>58.05750704271873</v>
       </c>
       <c r="J984" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K984" t="n">
         <v>-191.9364953941601</v>
@@ -44851,10 +44851,10 @@
         <v>10</v>
       </c>
       <c r="I985" t="n">
-        <v>33.19160704276669</v>
+        <v>33.19160704270985</v>
       </c>
       <c r="J985" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K985" t="n">
         <v>-191.9364953941601</v>
@@ -44895,10 +44895,10 @@
         <v>10</v>
       </c>
       <c r="I986" t="n">
-        <v>46.2211870427609</v>
+        <v>46.22118704270406</v>
       </c>
       <c r="J986" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K986" t="n">
         <v>-191.9364953941601</v>
@@ -44939,10 +44939,10 @@
         <v>10</v>
       </c>
       <c r="I987" t="n">
-        <v>60.04993704277695</v>
+        <v>60.0499370427201</v>
       </c>
       <c r="J987" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K987" t="n">
         <v>-191.9364953941601</v>
@@ -44983,10 +44983,10 @@
         <v>10</v>
       </c>
       <c r="I988" t="n">
-        <v>59.32542704277921</v>
+        <v>59.32542704272237</v>
       </c>
       <c r="J988" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K988" t="n">
         <v>-191.9364953941601</v>
@@ -45027,10 +45027,10 @@
         <v>10</v>
       </c>
       <c r="I989" t="n">
-        <v>59.61435704276141</v>
+        <v>59.61435704270457</v>
       </c>
       <c r="J989" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K989" t="n">
         <v>-191.9364953941601</v>
@@ -45071,10 +45071,10 @@
         <v>10</v>
       </c>
       <c r="I990" t="n">
-        <v>60.47604704278342</v>
+        <v>60.47604704272658</v>
       </c>
       <c r="J990" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K990" t="n">
         <v>-191.9364953941601</v>
@@ -45115,10 +45115,10 @@
         <v>10</v>
       </c>
       <c r="I991" t="n">
-        <v>30.66599704277451</v>
+        <v>30.66599704271766</v>
       </c>
       <c r="J991" t="n">
-        <v>-191.9974808870428</v>
+        <v>-191.9974808870427</v>
       </c>
       <c r="K991" t="n">
         <v>-191.9364953941601</v>

</xml_diff>

<commit_message>
Wed 12 Aug 2026 14:53:43 EDT
</commit_message>
<xml_diff>
--- a/machine_learning/injection/DDLUCJ-experiment-pipeline/repostprocess.xlsx
+++ b/machine_learning/injection/DDLUCJ-experiment-pipeline/repostprocess.xlsx
@@ -547,7 +547,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J2" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
@@ -557,11 +557,11 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>52.47680550405676</v>
+        <v>52.47680550408518</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
-        <v>-174.6675498512786</v>
+        <v>-174.6675498513071</v>
       </c>
       <c r="Q2" t="n">
         <v>-191.3796957923353</v>
@@ -604,7 +604,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J3" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
@@ -614,11 +614,11 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>65.15510550403292</v>
+        <v>65.15510550406134</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
-        <v>-161.9892498513025</v>
+        <v>-161.9892498513309</v>
       </c>
       <c r="Q3" t="n">
         <v>-178.7013957923591</v>
@@ -661,7 +661,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J4" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
@@ -671,11 +671,11 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>78.73617550404788</v>
+        <v>78.7361755040763</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
-        <v>-148.4081798512875</v>
+        <v>-148.4081798513159</v>
       </c>
       <c r="Q4" t="n">
         <v>-165.1203257923441</v>
@@ -718,7 +718,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J5" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
@@ -728,11 +728,11 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>139.2698855040351</v>
+        <v>139.2698855040635</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
-        <v>-87.87446985130032</v>
+        <v>-87.87446985132874</v>
       </c>
       <c r="Q5" t="n">
         <v>-104.586615792357</v>
@@ -775,7 +775,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J6" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
@@ -785,11 +785,11 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>43.90380550404416</v>
+        <v>43.90380550407258</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
-        <v>-183.2405498512912</v>
+        <v>-183.2405498513197</v>
       </c>
       <c r="Q6" t="n">
         <v>-199.9526957923479</v>
@@ -832,7 +832,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J7" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
@@ -842,11 +842,11 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>148.2584255040535</v>
+        <v>148.258425504082</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
-        <v>-78.88592985128184</v>
+        <v>-78.88592985131027</v>
       </c>
       <c r="Q7" t="n">
         <v>-95.59807579233848</v>
@@ -889,7 +889,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J8" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
@@ -899,11 +899,11 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>18.866835504042</v>
+        <v>18.86683550407042</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
-        <v>-208.2775198512934</v>
+        <v>-208.2775198513218</v>
       </c>
       <c r="Q8" t="n">
         <v>-224.98966579235</v>
@@ -946,7 +946,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J9" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
@@ -956,11 +956,11 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>23.36074550404987</v>
+        <v>23.3607455040783</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
-        <v>-203.7836098512855</v>
+        <v>-203.7836098513139</v>
       </c>
       <c r="Q9" t="n">
         <v>-220.4957557923422</v>
@@ -1003,7 +1003,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J10" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
@@ -1013,11 +1013,11 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>21.7005355040385</v>
+        <v>21.70053550406692</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
-        <v>-205.4438198512969</v>
+        <v>-205.4438198513253</v>
       </c>
       <c r="Q10" t="n">
         <v>-222.1559657923535</v>
@@ -1060,7 +1060,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J11" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
@@ -1070,11 +1070,11 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>30.55316550404541</v>
+        <v>30.55316550407383</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
-        <v>-196.59118985129</v>
+        <v>-196.5911898513184</v>
       </c>
       <c r="Q11" t="n">
         <v>-213.3033357923466</v>
@@ -1117,7 +1117,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J12" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
@@ -1127,11 +1127,11 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>47.79220550403807</v>
+        <v>47.79220550406649</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
-        <v>-179.3521498512973</v>
+        <v>-179.3521498513257</v>
       </c>
       <c r="Q12" t="n">
         <v>-196.064295792354</v>
@@ -1174,7 +1174,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J13" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
@@ -1184,11 +1184,11 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>179.4641455040562</v>
+        <v>179.4641455040846</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
-        <v>-47.68020985127919</v>
+        <v>-47.68020985130761</v>
       </c>
       <c r="Q13" t="n">
         <v>-64.39235579233582</v>
@@ -1231,7 +1231,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J14" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
@@ -1241,11 +1241,11 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>14.21445550403178</v>
+        <v>14.2144555040602</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
-        <v>-212.9298998513036</v>
+        <v>-212.929899851332</v>
       </c>
       <c r="Q14" t="n">
         <v>-229.6420457923602</v>
@@ -1288,7 +1288,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J15" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
@@ -1298,11 +1298,11 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>15.06347550403575</v>
+        <v>15.06347550406417</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
-        <v>-212.0808798512996</v>
+        <v>-212.0808798513281</v>
       </c>
       <c r="Q15" t="n">
         <v>-228.7930257923563</v>
@@ -1345,7 +1345,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J16" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
@@ -1355,11 +1355,11 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>25.67708550404291</v>
+        <v>25.67708550407133</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
-        <v>-201.4672698512925</v>
+        <v>-201.4672698513209</v>
       </c>
       <c r="Q16" t="n">
         <v>-218.1794157923491</v>
@@ -1402,7 +1402,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J17" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
@@ -1412,11 +1412,11 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>24.43076550403589</v>
+        <v>24.43076550406431</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
-        <v>-202.7135898512995</v>
+        <v>-202.7135898513279</v>
       </c>
       <c r="Q17" t="n">
         <v>-219.4257357923561</v>
@@ -1459,7 +1459,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J18" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
@@ -1469,11 +1469,11 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>20.91291550405572</v>
+        <v>20.91291550408414</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
-        <v>-206.2314398512797</v>
+        <v>-206.2314398513081</v>
       </c>
       <c r="Q18" t="n">
         <v>-222.9435857923363</v>
@@ -1516,7 +1516,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J19" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="n">
@@ -1526,11 +1526,11 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>186.1767955040534</v>
+        <v>186.1767955040818</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
-        <v>-40.96755985128198</v>
+        <v>-40.9675598513104</v>
       </c>
       <c r="Q19" t="n">
         <v>-57.67970579233861</v>
@@ -1573,7 +1573,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J20" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
@@ -1583,11 +1583,11 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>13.307345504046</v>
+        <v>13.30734550407442</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
-        <v>-213.8370098512894</v>
+        <v>-213.8370098513178</v>
       </c>
       <c r="Q20" t="n">
         <v>-230.549155792346</v>
@@ -1630,7 +1630,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J21" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
@@ -1640,11 +1640,11 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>23.90818550404106</v>
+        <v>23.90818550406948</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
-        <v>-203.2361698512943</v>
+        <v>-203.2361698513228</v>
       </c>
       <c r="Q21" t="n">
         <v>-219.948315792351</v>
@@ -1687,7 +1687,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J22" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
@@ -1697,11 +1697,11 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>9.196335504043418</v>
+        <v>9.19633550407184</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
-        <v>-217.948019851292</v>
+        <v>-217.9480198513204</v>
       </c>
       <c r="Q22" t="n">
         <v>-234.6601657923486</v>
@@ -1744,7 +1744,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J23" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
@@ -1754,11 +1754,11 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>10.60261550404107</v>
+        <v>10.60261550406949</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
-        <v>-216.5417398512943</v>
+        <v>-216.5417398513227</v>
       </c>
       <c r="Q23" t="n">
         <v>-233.253885792351</v>
@@ -1801,7 +1801,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J24" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
@@ -1811,11 +1811,11 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>20.04067550404898</v>
+        <v>20.0406755040774</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
-        <v>-207.1036798512864</v>
+        <v>-207.1036798513148</v>
       </c>
       <c r="Q24" t="n">
         <v>-223.815825792343</v>
@@ -1858,7 +1858,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J25" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
@@ -1868,11 +1868,11 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>183.762785504058</v>
+        <v>183.7627855040864</v>
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
-        <v>-43.38156985127739</v>
+        <v>-43.38156985130581</v>
       </c>
       <c r="Q25" t="n">
         <v>-60.09371579233402</v>
@@ -1915,7 +1915,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J26" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
@@ -1925,11 +1925,11 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>17.26795550405313</v>
+        <v>17.26795550408156</v>
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
-        <v>-209.8763998512823</v>
+        <v>-209.8763998513107</v>
       </c>
       <c r="Q26" t="n">
         <v>-226.5885457923389</v>
@@ -1972,7 +1972,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J27" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
@@ -1982,11 +1982,11 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>53.58427550405054</v>
+        <v>53.58427550407896</v>
       </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="n">
-        <v>-173.5600798512849</v>
+        <v>-173.5600798513133</v>
       </c>
       <c r="Q27" t="n">
         <v>-190.2722257923415</v>
@@ -2029,7 +2029,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J28" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
@@ -2039,11 +2039,11 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>11.44283550405589</v>
+        <v>11.44283550408431</v>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
-        <v>-215.7015198512795</v>
+        <v>-215.7015198513079</v>
       </c>
       <c r="Q28" t="n">
         <v>-232.4136657923361</v>
@@ -2086,7 +2086,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J29" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
@@ -2096,11 +2096,11 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>40.65523550403327</v>
+        <v>40.65523550406169</v>
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="n">
-        <v>-186.4891198513021</v>
+        <v>-186.4891198513305</v>
       </c>
       <c r="Q29" t="n">
         <v>-203.2012657923588</v>
@@ -2143,7 +2143,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J30" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
@@ -2153,11 +2153,11 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>17.53118550405475</v>
+        <v>17.53118550408317</v>
       </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="n">
-        <v>-209.6131698512806</v>
+        <v>-209.6131698513091</v>
       </c>
       <c r="Q30" t="n">
         <v>-226.3253157923373</v>
@@ -2200,7 +2200,7 @@
         <v>-213.3436138098513</v>
       </c>
       <c r="J31" t="n">
-        <v>-213.116469454496</v>
+        <v>-213.1164694544959</v>
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
@@ -2210,11 +2210,11 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>155.510235504039</v>
+        <v>155.5102355040674</v>
       </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="n">
-        <v>-71.63411985129642</v>
+        <v>-71.63411985132484</v>
       </c>
       <c r="Q31" t="n">
         <v>-88.34626579235305</v>
@@ -7504,7 +7504,7 @@
         <v>4</v>
       </c>
       <c r="I122" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J122" t="n">
         <v>-56.20522331321214</v>
@@ -7525,7 +7525,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P122" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q122" t="n">
         <v>301.3675192665275</v>
@@ -7565,7 +7565,7 @@
         <v>4</v>
       </c>
       <c r="I123" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J123" t="n">
         <v>-56.20522331321214</v>
@@ -7586,7 +7586,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P123" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q123" t="n">
         <v>301.3675192665275</v>
@@ -7626,7 +7626,7 @@
         <v>4</v>
       </c>
       <c r="I124" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J124" t="n">
         <v>-56.20522331321214</v>
@@ -7647,7 +7647,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P124" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q124" t="n">
         <v>301.3675192665275</v>
@@ -7687,7 +7687,7 @@
         <v>4</v>
       </c>
       <c r="I125" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J125" t="n">
         <v>-56.20522331321214</v>
@@ -7708,7 +7708,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P125" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q125" t="n">
         <v>301.3675192665275</v>
@@ -7748,7 +7748,7 @@
         <v>4</v>
       </c>
       <c r="I126" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J126" t="n">
         <v>-56.20522331321214</v>
@@ -7769,7 +7769,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P126" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q126" t="n">
         <v>301.3675192665275</v>
@@ -7809,7 +7809,7 @@
         <v>4</v>
       </c>
       <c r="I127" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J127" t="n">
         <v>-56.20522331321214</v>
@@ -7830,7 +7830,7 @@
         <v>-3.216402433281473e-05</v>
       </c>
       <c r="P127" t="n">
-        <v>0.002214823119572884</v>
+        <v>0.002214823126678311</v>
       </c>
       <c r="Q127" t="n">
         <v>301.3674892665321</v>
@@ -7870,7 +7870,7 @@
         <v>4</v>
       </c>
       <c r="I128" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J128" t="n">
         <v>-56.20522331321214</v>
@@ -7891,7 +7891,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P128" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q128" t="n">
         <v>301.3675192665275</v>
@@ -7931,7 +7931,7 @@
         <v>4</v>
       </c>
       <c r="I129" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J129" t="n">
         <v>-56.20522331321214</v>
@@ -7952,7 +7952,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P129" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q129" t="n">
         <v>301.3675192665275</v>
@@ -7992,7 +7992,7 @@
         <v>4</v>
       </c>
       <c r="I130" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J130" t="n">
         <v>-56.20522331321214</v>
@@ -8013,7 +8013,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P130" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q130" t="n">
         <v>301.3675192665275</v>
@@ -8053,7 +8053,7 @@
         <v>4</v>
       </c>
       <c r="I131" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J131" t="n">
         <v>-56.20522331321214</v>
@@ -8074,7 +8074,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P131" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q131" t="n">
         <v>301.3675192665275</v>
@@ -8114,7 +8114,7 @@
         <v>4</v>
       </c>
       <c r="I132" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J132" t="n">
         <v>-56.20522331321214</v>
@@ -8135,7 +8135,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P132" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q132" t="n">
         <v>301.3675192665275</v>
@@ -8175,7 +8175,7 @@
         <v>4</v>
       </c>
       <c r="I133" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J133" t="n">
         <v>-56.20522331321214</v>
@@ -8196,7 +8196,7 @@
         <v>-2.216402350541102e-05</v>
       </c>
       <c r="P133" t="n">
-        <v>0.002224823120400288</v>
+        <v>0.002224823127505715</v>
       </c>
       <c r="Q133" t="n">
         <v>301.3674992665329</v>
@@ -8236,7 +8236,7 @@
         <v>4</v>
       </c>
       <c r="I134" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J134" t="n">
         <v>-56.20522331321214</v>
@@ -8257,7 +8257,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P134" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q134" t="n">
         <v>301.3675192665275</v>
@@ -8297,7 +8297,7 @@
         <v>4</v>
       </c>
       <c r="I135" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J135" t="n">
         <v>-56.20522331321214</v>
@@ -8318,7 +8318,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P135" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q135" t="n">
         <v>301.3675192665275</v>
@@ -8358,7 +8358,7 @@
         <v>4</v>
       </c>
       <c r="I136" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J136" t="n">
         <v>-56.20522331321214</v>
@@ -8379,7 +8379,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P136" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q136" t="n">
         <v>301.3675192665275</v>
@@ -8419,7 +8419,7 @@
         <v>4</v>
       </c>
       <c r="I137" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J137" t="n">
         <v>-56.20522331321214</v>
@@ -8440,7 +8440,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P137" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q137" t="n">
         <v>301.3675192665275</v>
@@ -8480,7 +8480,7 @@
         <v>4</v>
       </c>
       <c r="I138" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J138" t="n">
         <v>-56.20522331321214</v>
@@ -8501,7 +8501,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P138" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q138" t="n">
         <v>301.3675192665275</v>
@@ -8541,7 +8541,7 @@
         <v>4</v>
       </c>
       <c r="I139" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J139" t="n">
         <v>-56.20522331321214</v>
@@ -8562,7 +8562,7 @@
         <v>-3.216402433281473e-05</v>
       </c>
       <c r="P139" t="n">
-        <v>0.002214823119572884</v>
+        <v>0.002214823126678311</v>
       </c>
       <c r="Q139" t="n">
         <v>301.3674892665321</v>
@@ -8602,7 +8602,7 @@
         <v>4</v>
       </c>
       <c r="I140" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J140" t="n">
         <v>-56.20522331321214</v>
@@ -8623,7 +8623,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P140" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q140" t="n">
         <v>301.3675192665275</v>
@@ -8663,7 +8663,7 @@
         <v>4</v>
       </c>
       <c r="I141" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J141" t="n">
         <v>-56.20522331321214</v>
@@ -8684,7 +8684,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P141" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q141" t="n">
         <v>301.3675192665275</v>
@@ -8724,7 +8724,7 @@
         <v>4</v>
       </c>
       <c r="I142" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J142" t="n">
         <v>-56.20522331321214</v>
@@ -8745,7 +8745,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P142" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q142" t="n">
         <v>301.3675192665275</v>
@@ -8785,7 +8785,7 @@
         <v>4</v>
       </c>
       <c r="I143" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J143" t="n">
         <v>-56.20522331321214</v>
@@ -8806,7 +8806,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P143" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q143" t="n">
         <v>301.3675192665275</v>
@@ -8846,7 +8846,7 @@
         <v>4</v>
       </c>
       <c r="I144" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J144" t="n">
         <v>-56.20522331321214</v>
@@ -8867,7 +8867,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P144" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q144" t="n">
         <v>301.3675192665275</v>
@@ -8907,7 +8907,7 @@
         <v>4</v>
       </c>
       <c r="I145" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J145" t="n">
         <v>-56.20522331321214</v>
@@ -8928,7 +8928,7 @@
         <v>-1.216402267800731e-05</v>
       </c>
       <c r="P145" t="n">
-        <v>0.002234823121227691</v>
+        <v>0.002234823128333119</v>
       </c>
       <c r="Q145" t="n">
         <v>301.3675092665338</v>
@@ -8968,7 +8968,7 @@
         <v>4</v>
       </c>
       <c r="I146" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J146" t="n">
         <v>-56.20522331321214</v>
@@ -8989,7 +8989,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P146" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q146" t="n">
         <v>301.3675192665275</v>
@@ -9029,7 +9029,7 @@
         <v>4</v>
       </c>
       <c r="I147" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J147" t="n">
         <v>-56.20522331321214</v>
@@ -9050,7 +9050,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P147" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q147" t="n">
         <v>301.3675192665275</v>
@@ -9090,7 +9090,7 @@
         <v>4</v>
       </c>
       <c r="I148" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J148" t="n">
         <v>-56.20522331321214</v>
@@ -9111,7 +9111,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P148" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q148" t="n">
         <v>301.3675192665275</v>
@@ -9151,7 +9151,7 @@
         <v>4</v>
       </c>
       <c r="I149" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J149" t="n">
         <v>-56.20522331321214</v>
@@ -9172,7 +9172,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P149" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q149" t="n">
         <v>301.3675192665275</v>
@@ -9212,7 +9212,7 @@
         <v>4</v>
       </c>
       <c r="I150" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J150" t="n">
         <v>-56.20522331321214</v>
@@ -9233,7 +9233,7 @@
         <v>-2.164028956030961e-06</v>
       </c>
       <c r="P150" t="n">
-        <v>0.002244823114949668</v>
+        <v>0.002244823122055095</v>
       </c>
       <c r="Q150" t="n">
         <v>301.3675192665275</v>
@@ -9273,7 +9273,7 @@
         <v>4</v>
       </c>
       <c r="I151" t="n">
-        <v>-56.20530663517688</v>
+        <v>-56.20530663517687</v>
       </c>
       <c r="J151" t="n">
         <v>-56.20522331321214</v>
@@ -9294,7 +9294,7 @@
         <v>-3.216402433281473e-05</v>
       </c>
       <c r="P151" t="n">
-        <v>0.002214823119572884</v>
+        <v>0.002214823126678311</v>
       </c>
       <c r="Q151" t="n">
         <v>301.3674892665321</v>
@@ -9349,7 +9349,7 @@
         <v>0</v>
       </c>
       <c r="N152" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O152" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9410,7 +9410,7 @@
         <v>0</v>
       </c>
       <c r="N153" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O153" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9471,7 +9471,7 @@
         <v>0</v>
       </c>
       <c r="N154" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O154" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9532,7 +9532,7 @@
         <v>0</v>
       </c>
       <c r="N155" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O155" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9593,7 +9593,7 @@
         <v>0</v>
       </c>
       <c r="N156" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O156" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9654,7 +9654,7 @@
         <v>0</v>
       </c>
       <c r="N157" t="n">
-        <v>11.11979359664872</v>
+        <v>11.11979359665582</v>
       </c>
       <c r="O157" t="n">
         <v>-0.0001763174211077967</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="N158" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O158" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9776,7 +9776,7 @@
         <v>0</v>
       </c>
       <c r="N159" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O159" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9837,7 +9837,7 @@
         <v>0</v>
       </c>
       <c r="N160" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O160" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9898,7 +9898,7 @@
         <v>0</v>
       </c>
       <c r="N161" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O161" t="n">
         <v>-1.631742208019205e-05</v>
@@ -9959,7 +9959,7 @@
         <v>0</v>
       </c>
       <c r="N162" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O162" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10020,7 +10020,7 @@
         <v>0</v>
       </c>
       <c r="N163" t="n">
-        <v>11.11984359664575</v>
+        <v>11.11984359665286</v>
       </c>
       <c r="O163" t="n">
         <v>-0.0001263174240762055</v>
@@ -10081,7 +10081,7 @@
         <v>0</v>
       </c>
       <c r="N164" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O164" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10142,7 +10142,7 @@
         <v>0</v>
       </c>
       <c r="N165" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O165" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10203,7 +10203,7 @@
         <v>0</v>
       </c>
       <c r="N166" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O166" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10264,7 +10264,7 @@
         <v>0</v>
       </c>
       <c r="N167" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O167" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10325,7 +10325,7 @@
         <v>0</v>
       </c>
       <c r="N168" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O168" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10386,7 +10386,7 @@
         <v>0</v>
       </c>
       <c r="N169" t="n">
-        <v>11.11987359664823</v>
+        <v>11.11987359665534</v>
       </c>
       <c r="O169" t="n">
         <v>-9.631742159399437e-05</v>
@@ -10447,7 +10447,7 @@
         <v>0</v>
       </c>
       <c r="N170" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O170" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10508,7 +10508,7 @@
         <v>0</v>
       </c>
       <c r="N171" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O171" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10569,7 +10569,7 @@
         <v>0</v>
       </c>
       <c r="N172" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O172" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10630,7 +10630,7 @@
         <v>0</v>
       </c>
       <c r="N173" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O173" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10691,7 +10691,7 @@
         <v>0</v>
       </c>
       <c r="N174" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O174" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10752,7 +10752,7 @@
         <v>0</v>
       </c>
       <c r="N175" t="n">
-        <v>11.11990359664361</v>
+        <v>11.11990359665072</v>
       </c>
       <c r="O175" t="n">
         <v>-6.63174262172106e-05</v>
@@ -10813,7 +10813,7 @@
         <v>0</v>
       </c>
       <c r="N176" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O176" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10874,7 +10874,7 @@
         <v>0</v>
       </c>
       <c r="N177" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O177" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10935,7 +10935,7 @@
         <v>0</v>
       </c>
       <c r="N178" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O178" t="n">
         <v>-1.631742208019205e-05</v>
@@ -10996,7 +10996,7 @@
         <v>0</v>
       </c>
       <c r="N179" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O179" t="n">
         <v>-1.631742208019205e-05</v>
@@ -11057,7 +11057,7 @@
         <v>0</v>
       </c>
       <c r="N180" t="n">
-        <v>11.11995359664775</v>
+        <v>11.11995359665485</v>
       </c>
       <c r="O180" t="n">
         <v>-1.631742208019205e-05</v>
@@ -11118,7 +11118,7 @@
         <v>0</v>
       </c>
       <c r="N181" t="n">
-        <v>11.11983359664492</v>
+        <v>11.11983359665203</v>
       </c>
       <c r="O181" t="n">
         <v>-0.0001363174249036092</v>
@@ -54017,7 +54017,7 @@
         <v>0</v>
       </c>
       <c r="N902" t="n">
-        <v>133.8007811942816</v>
+        <v>133.8007811942532</v>
       </c>
       <c r="O902" t="inlineStr"/>
       <c r="P902" t="n">
@@ -54074,7 +54074,7 @@
         <v>0</v>
       </c>
       <c r="N903" t="n">
-        <v>30.60974119426874</v>
+        <v>30.60974119424031</v>
       </c>
       <c r="O903" t="inlineStr"/>
       <c r="P903" t="n">
@@ -54131,7 +54131,7 @@
         <v>0</v>
       </c>
       <c r="N904" t="n">
-        <v>68.95023119429311</v>
+        <v>68.95023119426469</v>
       </c>
       <c r="O904" t="inlineStr"/>
       <c r="P904" t="n">
@@ -54188,7 +54188,7 @@
         <v>0</v>
       </c>
       <c r="N905" t="n">
-        <v>18.92639119427031</v>
+        <v>18.92639119424189</v>
       </c>
       <c r="O905" t="inlineStr"/>
       <c r="P905" t="n">
@@ -54245,7 +54245,7 @@
         <v>0</v>
       </c>
       <c r="N906" t="n">
-        <v>2.261601194277318</v>
+        <v>2.261601194248897</v>
       </c>
       <c r="O906" t="inlineStr"/>
       <c r="P906" t="n">
@@ -54302,7 +54302,7 @@
         <v>0</v>
       </c>
       <c r="N907" t="n">
-        <v>211.3868211942815</v>
+        <v>211.3868211942531</v>
       </c>
       <c r="O907" t="inlineStr"/>
       <c r="P907" t="n">
@@ -54359,7 +54359,7 @@
         <v>0</v>
       </c>
       <c r="N908" t="n">
-        <v>10.55412119427501</v>
+        <v>10.55412119424659</v>
       </c>
       <c r="O908" t="inlineStr"/>
       <c r="P908" t="n">
@@ -54416,7 +54416,7 @@
         <v>0</v>
       </c>
       <c r="N909" t="n">
-        <v>14.47989119427007</v>
+        <v>14.47989119424165</v>
       </c>
       <c r="O909" t="inlineStr"/>
       <c r="P909" t="n">
@@ -54473,7 +54473,7 @@
         <v>0</v>
       </c>
       <c r="N910" t="n">
-        <v>0.2617111942697647</v>
+        <v>0.261711194241343</v>
       </c>
       <c r="O910" t="inlineStr"/>
       <c r="P910" t="n">
@@ -54530,7 +54530,7 @@
         <v>0</v>
       </c>
       <c r="N911" t="n">
-        <v>37.93545119427222</v>
+        <v>37.9354511942438</v>
       </c>
       <c r="O911" t="inlineStr"/>
       <c r="P911" t="n">
@@ -54587,7 +54587,7 @@
         <v>0</v>
       </c>
       <c r="N912" t="n">
-        <v>3.427621194276753</v>
+        <v>3.427621194248331</v>
       </c>
       <c r="O912" t="inlineStr"/>
       <c r="P912" t="n">
@@ -54644,7 +54644,7 @@
         <v>0</v>
       </c>
       <c r="N913" t="n">
-        <v>212.6960611942934</v>
+        <v>212.696061194265</v>
       </c>
       <c r="O913" t="inlineStr"/>
       <c r="P913" t="n">
@@ -54701,7 +54701,7 @@
         <v>0</v>
       </c>
       <c r="N914" t="n">
-        <v>7.347691194269146</v>
+        <v>7.347691194240724</v>
       </c>
       <c r="O914" t="inlineStr"/>
       <c r="P914" t="n">
@@ -54758,7 +54758,7 @@
         <v>0</v>
       </c>
       <c r="N915" t="n">
-        <v>9.420881194273534</v>
+        <v>9.420881194245112</v>
       </c>
       <c r="O915" t="inlineStr"/>
       <c r="P915" t="n">
@@ -54815,7 +54815,7 @@
         <v>0</v>
       </c>
       <c r="N916" t="n">
-        <v>11.76894119427629</v>
+        <v>11.76894119424787</v>
       </c>
       <c r="O916" t="inlineStr"/>
       <c r="P916" t="n">
@@ -54872,7 +54872,7 @@
         <v>0</v>
       </c>
       <c r="N917" t="n">
-        <v>32.74884119429089</v>
+        <v>32.74884119426247</v>
       </c>
       <c r="O917" t="inlineStr"/>
       <c r="P917" t="n">
@@ -54929,7 +54929,7 @@
         <v>0</v>
       </c>
       <c r="N918" t="n">
-        <v>4.544831194266408</v>
+        <v>4.544831194237986</v>
       </c>
       <c r="O918" t="inlineStr"/>
       <c r="P918" t="n">
@@ -54986,7 +54986,7 @@
         <v>0</v>
       </c>
       <c r="N919" t="n">
-        <v>200.1835611942795</v>
+        <v>200.1835611942511</v>
       </c>
       <c r="O919" t="inlineStr"/>
       <c r="P919" t="n">
@@ -55043,7 +55043,7 @@
         <v>0</v>
       </c>
       <c r="N920" t="n">
-        <v>7.42672119429244</v>
+        <v>7.426721194264019</v>
       </c>
       <c r="O920" t="inlineStr"/>
       <c r="P920" t="n">
@@ -55100,7 +55100,7 @@
         <v>0</v>
       </c>
       <c r="N921" t="n">
-        <v>45.91803119427595</v>
+        <v>45.91803119424753</v>
       </c>
       <c r="O921" t="inlineStr"/>
       <c r="P921" t="n">
@@ -55157,7 +55157,7 @@
         <v>0</v>
       </c>
       <c r="N922" t="n">
-        <v>6.13761119427636</v>
+        <v>6.137611194247938</v>
       </c>
       <c r="O922" t="inlineStr"/>
       <c r="P922" t="n">
@@ -55214,7 +55214,7 @@
         <v>0</v>
       </c>
       <c r="N923" t="n">
-        <v>2.020251194267075</v>
+        <v>2.020251194238654</v>
       </c>
       <c r="O923" t="inlineStr"/>
       <c r="P923" t="n">
@@ -55271,7 +55271,7 @@
         <v>0</v>
       </c>
       <c r="N924" t="n">
-        <v>16.2967811942849</v>
+        <v>16.29678119425648</v>
       </c>
       <c r="O924" t="inlineStr"/>
       <c r="P924" t="n">
@@ -55328,7 +55328,7 @@
         <v>0</v>
       </c>
       <c r="N925" t="n">
-        <v>146.2915411942731</v>
+        <v>146.2915411942447</v>
       </c>
       <c r="O925" t="inlineStr"/>
       <c r="P925" t="n">
@@ -55385,7 +55385,7 @@
         <v>0</v>
       </c>
       <c r="N926" t="n">
-        <v>6.89056119426823</v>
+        <v>6.890561194239808</v>
       </c>
       <c r="O926" t="inlineStr"/>
       <c r="P926" t="n">
@@ -55442,7 +55442,7 @@
         <v>0</v>
       </c>
       <c r="N927" t="n">
-        <v>1.144901194265913</v>
+        <v>1.144901194237491</v>
       </c>
       <c r="O927" t="inlineStr"/>
       <c r="P927" t="n">
@@ -55499,7 +55499,7 @@
         <v>0</v>
       </c>
       <c r="N928" t="n">
-        <v>12.42525119428706</v>
+        <v>12.42525119425864</v>
       </c>
       <c r="O928" t="inlineStr"/>
       <c r="P928" t="n">
@@ -55556,7 +55556,7 @@
         <v>0</v>
       </c>
       <c r="N929" t="n">
-        <v>6.624331194274191</v>
+        <v>6.624331194245769</v>
       </c>
       <c r="O929" t="inlineStr"/>
       <c r="P929" t="n">
@@ -55613,7 +55613,7 @@
         <v>0</v>
       </c>
       <c r="N930" t="n">
-        <v>3.770581194288525</v>
+        <v>3.770581194260103</v>
       </c>
       <c r="O930" t="inlineStr"/>
       <c r="P930" t="n">
@@ -55670,7 +55670,7 @@
         <v>0</v>
       </c>
       <c r="N931" t="n">
-        <v>206.3054711942698</v>
+        <v>206.3054711942414</v>
       </c>
       <c r="O931" t="inlineStr"/>
       <c r="P931" t="n">

</xml_diff>